<commit_message>
feat: separar por cliente, subir XML desde el chat y evaluaciones de la IA
</commit_message>
<xml_diff>
--- a/salida/reporte_cfdi.xlsx
+++ b/salida/reporte_cfdi.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen por proveedor" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Detalle'!$A$1:$K$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Detalle'!$A$1:$M$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -443,10 +443,12 @@
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,20 +489,30 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>RFC receptor</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre receptor</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Serie</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Folio</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Moneda</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Archivo</t>
         </is>
@@ -536,20 +548,30 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>A1012</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>factura_15.xml</t>
         </is>
@@ -585,20 +607,30 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>A1013</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>factura_16.xml</t>
         </is>
@@ -634,20 +666,30 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>A1015</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>factura_18.xml</t>
         </is>
@@ -683,20 +725,30 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>A1004</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>factura_06.xml</t>
         </is>
@@ -732,20 +784,30 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>A1008</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>factura_10.xml</t>
         </is>
@@ -781,20 +843,30 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>A1009</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>factura_12.xml</t>
         </is>
@@ -830,20 +902,30 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>A1014</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>factura_17.xml</t>
         </is>
@@ -879,20 +961,30 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>A1011</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>factura_14.xml</t>
         </is>
@@ -928,20 +1020,30 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>A1002</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>factura_03.xml</t>
         </is>
@@ -977,20 +1079,30 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>A1005</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>factura_07.xml</t>
         </is>
@@ -1026,20 +1138,30 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>A1001</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>factura_02.xml</t>
         </is>
@@ -1075,20 +1197,30 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>A1003</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>factura_05.xml</t>
         </is>
@@ -1124,20 +1256,30 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>A1000</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>factura_01.xml</t>
         </is>
@@ -1173,27 +1315,37 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
+          <t>CDE150101AB1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>CLIENTE DEMO</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>A1010</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>factura_13.xml</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K15"/>
+  <autoFilter ref="A1:M15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cambio de formato en los reportes de acuerdo a los colores de la empresa
</commit_message>
<xml_diff>
--- a/salida/reporte_cfdi.xlsx
+++ b/salida/reporte_cfdi.xlsx
@@ -11,7 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen por proveedor" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Detalle'!$A$1:$M$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Detalle'!$A$4:$M$18</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Detalle'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resumen por proveedor'!$A$4:$F$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Resumen por proveedor'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,10 +24,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,10 +36,35 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001F1F1F"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F1F1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,11 +73,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="001F1F1F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6F4EF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -57,17 +90,72 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00C9A13B"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00DDD8CC"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="00C9A13B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C9A13B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,1144 +518,1240 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C9A13B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="41" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Revisión de CFDI · Detalle de facturas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generado el 20/10/2026 22:05 · Cliente: Todos · 14 facturas</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>UUID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>RFC emisor</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Nombre emisor</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>IVA trasladado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>RFC receptor</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Nombre receptor</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Serie</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Folio</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Moneda</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Archivo</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>D1711CBD-2106-119E-C40D-31B5397A7623</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>MAGR850714HJ3</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>MARIO GARCIA RUIZ</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D5" s="7" t="n">
         <v>46267.70555555556</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E5" s="8" t="n">
         <v>2046.48</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F5" s="8" t="n">
         <v>327.44</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G5" s="8" t="n">
         <v>2373.92</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>A1012</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>factura_15.xml</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>78549014-6DED-C86A-9F4F-B02BB7A1774F</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>CON170405PL9</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>CONSTRUCTORA ATEMAJAC DEMO</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D6" s="10" t="n">
         <v>46270.66388888889</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E6" s="11" t="n">
         <v>32463.28</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F6" s="11" t="n">
         <v>5194.12</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G6" s="11" t="n">
         <v>37657.4</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>A1013</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>factura_16.xml</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>8BAE8E66-FA97-002C-FCBA-D167F5A9CA5F</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>PAP180312KL4</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>PAPELERIA DEL BAJIO DEMO</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D7" s="7" t="n">
         <v>46274.68402777778</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E7" s="8" t="n">
         <v>34539.77</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F7" s="8" t="n">
         <v>5526.36</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G7" s="8" t="n">
         <v>40066.13</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>A1015</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>factura_18.xml</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>ADEC6F11-7D83-6E77-AF67-D461E4163207</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>SLT200915QW2</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>SERVICIOS LOGISTICOS TAPATIOS DEMO</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D8" s="10" t="n">
         <v>46276.47569444445</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E8" s="11" t="n">
         <v>1391.7</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F8" s="11" t="n">
         <v>222.67</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G8" s="11" t="n">
         <v>1614.37</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K8" s="9" t="inlineStr">
         <is>
           <t>A1004</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>factura_06.xml</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>7608D942-5D11-1A9D-5E6C-9992B5FB12E0</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>TEC190101MN8</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>TECNOLOGIA EMPRESARIAL OCCIDENTE DEMO</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D9" s="7" t="n">
         <v>46279.39236111111</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E9" s="8" t="n">
         <v>2016.46</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F9" s="8" t="n">
         <v>322.63</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G9" s="8" t="n">
         <v>2339.09</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>A1008</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>factura_10.xml</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>1DCF884C-DE02-79E1-7F9A-C0988DF05F25</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>ALI210622RT5</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>ALIMENTOS SELECTOS ZAPOPAN DEMO</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D10" s="10" t="n">
         <v>46279.70208333333</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E10" s="11" t="n">
         <v>42859.18</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G10" s="11" t="n">
         <v>42859.18</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J10" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K10" s="9" t="inlineStr">
         <is>
           <t>A1009</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L10" s="9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M10" s="9" t="inlineStr">
         <is>
           <t>factura_12.xml</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>B3618E1C-A06D-7A69-1F3C-42B2E2CBBB93</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>CON170405PL9</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>CONSTRUCTORA ATEMAJAC DEMO</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D11" s="7" t="n">
         <v>46280.77083333334</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E11" s="8" t="n">
         <v>11643.92</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F11" s="8" t="n">
         <v>1863.03</v>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G11" s="8" t="n">
         <v>13506.95</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>A1014</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>factura_17.xml</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>7AAC319F-FB75-9E0F-ED1D-9D1690624FE3</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>MAGR850714HJ3</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>MARIO GARCIA RUIZ</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D12" s="10" t="n">
         <v>46282.70208333333</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E12" s="11" t="n">
         <v>40667.12</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F12" s="11" t="n">
         <v>6506.74</v>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G12" s="11" t="n">
         <v>47173.86</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J12" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K12" s="9" t="inlineStr">
         <is>
           <t>A1011</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L12" s="9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M12" s="9" t="inlineStr">
         <is>
           <t>factura_14.xml</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>C0433CBD-7DAB-E929-C4A3-34BFC6CD75E9</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>PAP180312KL4</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>PAPELERIA DEL BAJIO DEMO</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D13" s="7" t="n">
         <v>46290.72777777778</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E13" s="8" t="n">
         <v>40569.24</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F13" s="8" t="n">
         <v>6491.08</v>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G13" s="8" t="n">
         <v>47060.32</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>A1002</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>factura_03.xml</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>5B4C8012-EDE7-BD0C-FFB8-8309FADB8908</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>SLT200915QW2</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>SERVICIOS LOGISTICOS TAPATIOS DEMO</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D14" s="10" t="n">
         <v>46291.61597222222</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E14" s="11" t="n">
         <v>12708.84</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F14" s="11" t="n">
         <v>2033.41</v>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="G14" s="11" t="n">
         <v>14742.25</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J14" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K14" s="9" t="inlineStr">
         <is>
           <t>A1005</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L14" s="9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M14" s="9" t="inlineStr">
         <is>
           <t>factura_07.xml</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>6BAD6BE2-8E7A-A6E9-9F19-950499DD251D</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>PAP180312KL4</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>PAPELERIA DEL BAJIO DEMO</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D15" s="7" t="n">
         <v>46291.73263888889</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E15" s="8" t="n">
         <v>11377.87</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F15" s="8" t="n">
         <v>1820.46</v>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G15" s="8" t="n">
         <v>13198.33</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>A1001</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>factura_02.xml</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>49889310-1C59-3AF5-14AA-4E719D3C7DEC</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>SLT200915QW2</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>SERVICIOS LOGISTICOS TAPATIOS DEMO</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D16" s="10" t="n">
         <v>46292.39444444444</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E16" s="11" t="n">
         <v>12162.89</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F16" s="11" t="n">
         <v>1946.06</v>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="G16" s="11" t="n">
         <v>14108.95</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J16" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K16" s="9" t="inlineStr">
         <is>
           <t>A1003</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M16" s="9" t="inlineStr">
         <is>
           <t>factura_05.xml</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>A5AEC797-8306-D03B-F38B-2FFC80A4DF5A</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>PAP180312KL4</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>PAPELERIA DEL BAJIO DEMO</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D17" s="7" t="n">
         <v>46293.41388888889</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E17" s="8" t="n">
         <v>6466.5</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F17" s="8" t="n">
         <v>1034.64</v>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="G17" s="8" t="n">
         <v>7501.14</v>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>A1000</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
         <is>
           <t>factura_01.xml</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>65ED0DE4-7DB4-304D-E01C-683E99A46DF0</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>ALI210622RT5</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>ALIMENTOS SELECTOS ZAPOPAN DEMO</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D18" s="10" t="n">
         <v>46295.67777777778</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E18" s="11" t="n">
         <v>36219.42</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F18" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="G18" s="11" t="n">
         <v>36219.42</v>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>CDE150101AB1</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I18" s="9" t="inlineStr">
         <is>
           <t>CLIENTE DEMO</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J18" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K18" s="9" t="inlineStr">
         <is>
           <t>A1010</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L18" s="9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M18" s="9" t="inlineStr">
         <is>
           <t>factura_13.xml</t>
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="13">
+        <f>SUM(E5:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="13">
+        <f>SUM(F5:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="13">
+        <f>SUM(G5:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="12" t="n"/>
+      <c r="L19" s="12" t="n"/>
+      <c r="M19" s="12" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M15"/>
+  <autoFilter ref="A4:M18"/>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="5" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LRevisión de CFDI · Detalle de facturas&amp;RPágina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C9A13B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Revisión de CFDI · Resumen por proveedor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generado el 20/10/2026 22:05 · Cliente: Todos · 6 proveedores · de mayor a menor total facturado</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>RFC emisor</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Nombre emisor</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Facturas</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>IVA trasladado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Total facturado</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>PAP180312KL4</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>PAPELERIA DEL BAJIO DEMO</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D5" s="8" t="n">
         <v>92953.38</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E5" s="8" t="n">
         <v>14872.54</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F5" s="8" t="n">
         <v>107825.92</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>ALI210622RT5</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>ALIMENTOS SELECTOS ZAPOPAN DEMO</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C6" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D6" s="11" t="n">
         <v>79078.60000000001</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F6" s="11" t="n">
         <v>79078.60000000001</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>CON170405PL9</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>CONSTRUCTORA ATEMAJAC DEMO</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C7" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D7" s="8" t="n">
         <v>44107.2</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E7" s="8" t="n">
         <v>7057.15</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F7" s="8" t="n">
         <v>51164.35</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>MAGR850714HJ3</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>MARIO GARCIA RUIZ</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C8" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D8" s="11" t="n">
         <v>42713.6</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E8" s="11" t="n">
         <v>6834.18</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F8" s="11" t="n">
         <v>49547.78</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>SLT200915QW2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>SERVICIOS LOGISTICOS TAPATIOS DEMO</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D9" s="8" t="n">
         <v>26263.43</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E9" s="8" t="n">
         <v>4202.14</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F9" s="8" t="n">
         <v>30465.57</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>TEC190101MN8</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>TECNOLOGIA EMPRESARIAL OCCIDENTE DEMO</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C10" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D10" s="11" t="n">
         <v>2016.46</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E10" s="11" t="n">
         <v>322.63</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F10" s="11" t="n">
         <v>2339.09</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4">
-        <f>SUM(C2:C7)</f>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="16">
+        <f>SUM(C5:C10)</f>
         <v/>
       </c>
-      <c r="D8" s="5">
-        <f>SUM(D2:D7)</f>
+      <c r="D11" s="13">
+        <f>SUM(D5:D10)</f>
         <v/>
       </c>
-      <c r="E8" s="5">
-        <f>SUM(E2:E7)</f>
+      <c r="E11" s="13">
+        <f>SUM(E5:E10)</f>
         <v/>
       </c>
-      <c r="F8" s="5">
-        <f>SUM(F2:F7)</f>
+      <c r="F11" s="13">
+        <f>SUM(F5:F10)</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:F10"/>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LRevisión de CFDI · Resumen por proveedor&amp;RPágina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
el reto y el bot ya no comparten log ni Excel
</commit_message>
<xml_diff>
--- a/salida/reporte_cfdi.xlsx
+++ b/salida/reporte_cfdi.xlsx
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado el 20/10/2026 22:05 · Cliente: Todos · 14 facturas</t>
+          <t>Generado el 20/10/2026 23:11 · Cliente: Todos · Carpeta: cfdis · 14 facturas</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -1531,7 +1531,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado el 20/10/2026 22:05 · Cliente: Todos · 6 proveedores · de mayor a menor total facturado</t>
+          <t>Generado el 20/10/2026 23:11 · Cliente: Todos · Carpeta: cfdis · 6 proveedores · de mayor a menor total facturado</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>

</xml_diff>

<commit_message>
resolucion de los acentos en la salida
</commit_message>
<xml_diff>
--- a/salida/reporte_cfdi.xlsx
+++ b/salida/reporte_cfdi.xlsx
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado el 20/10/2026 23:11 · Cliente: Todos · Carpeta: cfdis · 14 facturas</t>
+          <t>Generado el 21/10/2026 09:33 · Cliente: Todos · Carpeta: cfdis · 14 facturas</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -1531,7 +1531,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado el 20/10/2026 23:11 · Cliente: Todos · Carpeta: cfdis · 6 proveedores · de mayor a menor total facturado</t>
+          <t>Generado el 21/10/2026 09:33 · Cliente: Todos · Carpeta: cfdis · 6 proveedores · de mayor a menor total facturado</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>

</xml_diff>